<commit_message>
Add Swagger UI, Cucumber BDD tests, scripts, and README
- Replace Testcontainers with H2 for tests
- Add SpringDoc OpenAPI (Swagger UI) with endpoint annotations
- Add Cucumber/Gherkin BDD tests covering all CRUD scenarios (15 scenarios)
- Add start/test/demo scripts for Linux/Mac (.sh) and Windows (.bat)
- Add Gradle wrapper
- Add comprehensive README.md

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/api-documentation.xlsx
+++ b/docs/api-documentation.xlsx
@@ -275,13 +275,13 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="2.3359375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="7.72265625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="16.53515625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="19.265625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="27.38671875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="47.41015625" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="13.28125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="2.0078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="7.0625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="18.48828125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="25.62890625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="44.9453125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="13.1328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,10 +440,10 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="9.12109375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="9.8125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="9.04296875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="14.2578125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="8.8984375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="9.4453125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="8.27734375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.73828125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>